<commit_message>
Remove HKUST; keep Charles Darwin in OK pending partner confirmation
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EZa6h9SpqLeB7ZbHz6KiwN
</commit_message>
<xml_diff>
--- a/curriculum_mapping_2026-27/CurriculumMapping_Geo_2_ReviewEntry_NOT_met.xlsx
+++ b/curriculum_mapping_2026-27/CurriculumMapping_Geo_2_ReviewEntry_NOT_met.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Geography BA'!$A$1:$K$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Geography BSc'!$A$1:$K$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Geography BSc'!$A$1:$K$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Rows removed (not usable)'!$A$1:$K$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Candidates'!$A$1:$K$10</definedName>
   </definedNames>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -586,16 +586,16 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Charles Darwin University</t>
+          <t>City University of Hong Kong</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Geography BSc</t>
+          <t>Geography BA</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>0</v>
@@ -603,53 +603,20 @@
       <c r="E6" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Not on the confirmed partner list (Summer 2026 Final)</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="n"/>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Not enough modules after 2026/27 term check: 2 confirmed + 0 unverified, 4 needed</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Semester A</t>
+        </is>
+      </c>
       <c r="H6" s="3" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>City University of Hong Kong</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Not enough modules after 2026/27 term check: 2 confirmed + 0 unverified, 4 needed</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>Semester A</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="I7" s="3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -855,7 +822,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -981,432 +948,8 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Charles Darwin University — Australia</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Geography BSc</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>SOES214 CHANGING ENVIRONMENTS</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>ENV101 Earth Systems</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Level 1</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>2026/27 module/catalogue verified; exact semester not publicly specified</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>Host: https://www.cdu.edu.au/international/learning-abroad/inbound-australia/student-exchange | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>Original row</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Charles Darwin University — Australia</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Geography BSc</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>SOES214 CHANGING ENVIRONMENTS</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>ENV103 Environmental Issues</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Level 1</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>2026/27 module/catalogue verified; exact semester not publicly specified</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>Host: https://www.cdu.edu.au/international/learning-abroad/inbound-australia/student-exchange | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>Original row</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Charles Darwin University — Australia</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Geography BSc</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>SOES214 CHANGING ENVIRONMENTS</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>ENV201 Introductory Ecology</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Level 2</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>2026/27 module/catalogue verified; exact semester not publicly specified</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="n"/>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>Host: https://www.cdu.edu.au/international/learning-abroad/inbound-australia/student-exchange | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
-        </is>
-      </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>Original row</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Charles Darwin University — Australia</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Geography BSc</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>ENV202 Introductory Remote Sensing</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Level 2</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>2026/27 module/catalogue verified; exact semester not publicly specified</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="n"/>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>Host: https://www.cdu.edu.au/international/learning-abroad/inbound-australia/student-exchange | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>Original row</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Charles Darwin University — Australia</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Geography BSc</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>SOES214 CHANGING ENVIRONMENTS</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>ENV208 Geographical Information Systems and Spatial Thinking</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Level 2</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>2026/27 module/catalogue verified; exact semester not publicly specified</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="n"/>
-      <c r="J7" s="3" t="inlineStr">
-        <is>
-          <t>Host: https://www.cdu.edu.au/international/learning-abroad/inbound-australia/student-exchange | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
-        </is>
-      </c>
-      <c r="K7" s="3" t="inlineStr">
-        <is>
-          <t>Original row</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Charles Darwin University — Australia</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Geography BSc</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>SOES213 GEOGRAPHICAL DATA ANALYSIS AND PROCESSING</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>ENV306 Environmental Monitoring and Modelling</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>Level 3</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>2026/27 module/catalogue verified; exact semester not publicly specified</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="n"/>
-      <c r="J8" s="3" t="inlineStr">
-        <is>
-          <t>Host: https://www.cdu.edu.au/international/learning-abroad/inbound-australia/student-exchange | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
-        </is>
-      </c>
-      <c r="K8" s="3" t="inlineStr">
-        <is>
-          <t>Original row</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Charles Darwin University — Australia</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Geography BSc</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>SOES280 HYDROCLIMATE</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>ENV313 Hydrology and Catchment Processes</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>Level 3</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>2026/27 module/catalogue verified; exact semester not publicly specified</t>
-        </is>
-      </c>
-      <c r="I9" s="3" t="n"/>
-      <c r="J9" s="3" t="inlineStr">
-        <is>
-          <t>Host: https://www.cdu.edu.au/international/learning-abroad/inbound-australia/student-exchange | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
-        </is>
-      </c>
-      <c r="K9" s="3" t="inlineStr">
-        <is>
-          <t>Original row</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Charles Darwin University — Australia</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Geography BSc</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>SOES214 CHANGING ENVIRONMENTS</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>ENV318 Solving Real-World Spatial Problems</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>Level 3</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>2026/27 module/catalogue verified; exact semester not publicly specified</t>
-        </is>
-      </c>
-      <c r="I10" s="3" t="n"/>
-      <c r="J10" s="3" t="inlineStr">
-        <is>
-          <t>Host: https://www.cdu.edu.au/international/learning-abroad/inbound-australia/student-exchange | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
-        </is>
-      </c>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
-          <t>Original row</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K10"/>
+  <autoFilter ref="A1:K2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Infer missing terms from previous years (flagged lilac); CDU 2027 availability checked
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EZa6h9SpqLeB7ZbHz6KiwN
</commit_message>
<xml_diff>
--- a/curriculum_mapping_2026-27/CurriculumMapping_Geo_2_ReviewEntry_NOT_met.xlsx
+++ b/curriculum_mapping_2026-27/CurriculumMapping_Geo_2_ReviewEntry_NOT_met.xlsx
@@ -49,7 +49,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -74,6 +74,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00E4DFEC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00F8CBAD"/>
       </patternFill>
     </fill>
@@ -90,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -104,6 +109,9 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -495,7 +503,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Updated 5 Oct 2026 (deep check). Only modules running in the partner exchange period count: UoL Semester 1 partners = Fall 2026 / Term 1 / Semester A; UoL Semester 2 partners = Semester 1 2027 (Australia), Trimester 1 2027 (Wellington), Semester 2 2026-27 (Netherlands); XJTLU, HKUST, SNU and Calgary accept either semester. Amber rows = term could not be verified (timetable behind login / captcha / not yet published). Green rows = modules added Oct 2026 from the 2026/27 timetables. UoL matches on added rows are suggestions for department review.</t>
+          <t>Updated 5 Oct 2026 (deep check). Only modules running in the partner exchange period count: UoL Semester 1 partners = Fall 2026 / Term 1 / Semester A; UoL Semester 2 partners = Semester 1 2027 (Australia), Trimester 1 2027 (Wellington), Semester 2 2026-27 (Netherlands); XJTLU, HKUST, SNU and Calgary accept either semester. Amber rows = term could not be verified (timetable behind login / captcha / not yet published). Green rows = modules added Oct 2026 from the 2026/27 timetables. Lilac rows = term INFERRED from previous years or the usual offering pattern (TERM LIKELY / TERM FROM PREVIOUS YEAR) because the 2026/27 timetable is not yet published - confirm when available. UoL matches on added rows are suggestions for department review.</t>
         </is>
       </c>
     </row>
@@ -896,53 +904,53 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Australian Catholic University — Australia</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>Geography BSc</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>SOES214 CHANGING ENVIRONMENTS</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>Level 5</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>GEOG218 Natural Disasters: Risk, Response and Resilience (10 CP)</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>Level 2</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>Semester 1 2026, online scheduled (2027 not confirmed)</t>
         </is>
       </c>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="I2" s="6" t="n"/>
+      <c r="J2" s="6" t="inlineStr">
         <is>
           <t>Host: https://www.acu.edu.au/handbook/handbook-2026/major/geography-environment-and-society | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K2" s="6" t="inlineStr">
         <is>
           <t>Original row; TERM LIKELY (2026/27 timetable not yet published or pattern only): Semester 1 2026, online scheduled (2027 not confirmed) [https://www.acu.edu.au/handbook/handbook-2026/]</t>
         </is>
@@ -1034,212 +1042,212 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>Australian Catholic University — Australia</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>Geography BSc</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>SOES214 CHANGING ENVIRONMENTS</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>Level 5</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>GEOG110 Exploring Natural Environments (10 CP)</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr">
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>Level 1</t>
         </is>
       </c>
-      <c r="G2" s="6" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="H2" s="6" t="inlineStr">
+      <c r="H2" s="7" t="inlineStr">
         <is>
           <t>Semester 2 (2026)</t>
         </is>
       </c>
-      <c r="I2" s="6" t="n"/>
-      <c r="J2" s="6" t="inlineStr">
+      <c r="I2" s="7" t="n"/>
+      <c r="J2" s="7" t="inlineStr">
         <is>
           <t>Host: https://www.acu.edu.au/handbook/handbook-2026/major/geography-environment-and-society | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
         </is>
       </c>
-      <c r="K2" s="6" t="inlineStr">
+      <c r="K2" s="7" t="inlineStr">
         <is>
           <t>Original row; Wrong term for partner semester (Semester 1)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Australian Catholic University — Australia</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>Geography BSc</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>SOES280 HYDROCLIMATE</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>Level 5</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>GEOG216 Climate Change: Past, Present and Future (10 CP)</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>Level 2</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>Not listed in 2026 Geography, Environment and Society unit availability</t>
         </is>
       </c>
-      <c r="I3" s="6" t="n"/>
-      <c r="J3" s="6" t="inlineStr">
+      <c r="I3" s="7" t="n"/>
+      <c r="J3" s="7" t="inlineStr">
         <is>
           <t>Host: https://www.acu.edu.au/handbook/handbook-2026/major/geography-environment-and-society | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
         </is>
       </c>
-      <c r="K3" s="6" t="inlineStr">
+      <c r="K3" s="7" t="inlineStr">
         <is>
           <t>Original row; Workbook semester note says not currently offered</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Australian Catholic University — Australia</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Geography BSc</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>SOES280 HYDROCLIMATE</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>Level 5</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>GEOG311 Catchments to Coasts (10 CP)</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>Level 3</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>Semester 2 (2026)</t>
         </is>
       </c>
-      <c r="I4" s="6" t="n"/>
-      <c r="J4" s="6" t="inlineStr">
+      <c r="I4" s="7" t="n"/>
+      <c r="J4" s="7" t="inlineStr">
         <is>
           <t>Host: https://www.acu.edu.au/handbook/handbook-2026/major/geography-environment-and-society | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
         </is>
       </c>
-      <c r="K4" s="6" t="inlineStr">
+      <c r="K4" s="7" t="inlineStr">
         <is>
           <t>Original row; Wrong term for partner semester (Semester 1)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Australian Catholic University — Australia</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Geography BSc</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>Level 5</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>GEOG312 Mapping for a Complex World (10 CP)</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>Level 3</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>Not listed in 2026 Geography, Environment and Society unit availability</t>
         </is>
       </c>
-      <c r="I5" s="6" t="n"/>
-      <c r="J5" s="6" t="inlineStr">
+      <c r="I5" s="7" t="n"/>
+      <c r="J5" s="7" t="inlineStr">
         <is>
           <t>Host: https://www.acu.edu.au/handbook/handbook-2026/major/geography-environment-and-society | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
         </is>
       </c>
-      <c r="K5" s="6" t="inlineStr">
+      <c r="K5" s="7" t="inlineStr">
         <is>
           <t>Original row; Workbook semester note says not currently offered</t>
         </is>

</xml_diff>

<commit_message>
CityU BA: Semester A PIA courses added (marked Full), moved to OK
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EZa6h9SpqLeB7ZbHz6KiwN
</commit_message>
<xml_diff>
--- a/curriculum_mapping_2026-27/CurriculumMapping_Geo_2_ReviewEntry_NOT_met.xlsx
+++ b/curriculum_mapping_2026-27/CurriculumMapping_Geo_2_ReviewEntry_NOT_met.xlsx
@@ -11,13 +11,11 @@
     <sheet name="Geography BA" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Geography BSc" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Rows removed (not usable)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Candidates" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Geography BA'!$A$1:$K$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Geography BA'!$A$1:$K$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Geography BSc'!$A$1:$K$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Rows removed (not usable)'!$A$1:$K$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Candidates'!$A$1:$K$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -479,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -591,43 +589,6 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>City University of Hong Kong</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Not enough modules after 2026/27 term check: 2 confirmed + 0 unverified, 4 needed</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>Semester A</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="I6" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -639,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -712,114 +673,8 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>City University of Hong Kong — Hong Kong (SAR)</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>SOES225 THEMES IN URBAN GEOGRAPHY</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>GE2244 The Hidden City: Space, Power and Social Processes in Hong Kong (3 credits)</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Level 2</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>Semesters A and B (2026/27)</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>Host: https://www.cityu.edu.hk/class/exchange/content/inbound/course_2627.aspx?dept=SS&amp;sem=A | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr">
-        <is>
-          <t>Original row; TERM VERIFIED Oct 2026: Semesters A and B (2026/27)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>City University of Hong Kong — Hong Kong (SAR)</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>SOES225 THEMES IN URBAN GEOGRAPHY</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>PIA3921 Urban and Social Policy (3 credits)</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Level 1</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Semester A</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>Host: https://www.cityu.edu.hk/class/exchange/content/inbound/course_2627.aspx?dept=SS&amp;sem=A | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>Original row</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K3"/>
+  <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1257,566 +1112,4 @@
   <autoFilter ref="A1:K5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="58" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="70" customWidth="1" min="10" max="10"/>
-    <col width="60" customWidth="1" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>University name and country</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>Programme title</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>UoL module code and title</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>UoL module level</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>Host uni module code and title</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>Host uni module level</t>
-        </is>
-      </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>Core or optional</t>
-        </is>
-      </c>
-      <c r="H1" s="5" t="inlineStr">
-        <is>
-          <t>Semester</t>
-        </is>
-      </c>
-      <c r="I1" s="5" t="inlineStr">
-        <is>
-          <t>CB approval</t>
-        </is>
-      </c>
-      <c r="J1" s="5" t="inlineStr">
-        <is>
-          <t>Evidence / source URL</t>
-        </is>
-      </c>
-      <c r="K1" s="5" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>City University of Hong Kong — Hong Kong (SAR)</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>SOES275 SOCIAL AND CULTURAL GEOGRAPHIES (suggested)</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>GE2215 Tourism, Development and Society (3 credit units)</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>Level 2</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>CANDIDATE - on 2026/27 inbound exchange list (Semester B list); Semester A list not yet published - confirm Semester A</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="n"/>
-      <c r="J2" s="4" t="inlineStr">
-        <is>
-          <t>Host: https://banweb.cityu.edu.hk/pls/PROD/hwiecrselis_cityu.P_Main</t>
-        </is>
-      </c>
-      <c r="K2" s="4" t="inlineStr">
-        <is>
-          <t>Candidate - Semester A to confirm</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>City University of Hong Kong — Hong Kong (SAR)</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>SOES225 THEMES IN URBAN GEOGRAPHY (suggested)</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>PIA3310 Smart Government and Sustainable Cities (3 credit units)</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Level 3</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>CANDIDATE - on 2026/27 inbound exchange list (Semester B list); Semester A list not yet published - confirm Semester A</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="n"/>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>Host: https://banweb.cityu.edu.hk/pls/PROD/hwiecrselis_cityu.P_Main</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>Candidate - Semester A to confirm</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>City University of Hong Kong — Hong Kong (SAR)</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>SOES225 THEMES IN URBAN GEOGRAPHY (suggested)</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>PIA3503 Urbanization and Health Management (3 credit units)</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Level 3</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>CANDIDATE - on 2026/27 inbound exchange list (Semester B list); Semester A list not yet published - confirm Semester A</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="n"/>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>Host: https://banweb.cityu.edu.hk/pls/PROD/hwiecrselis_cityu.P_Main</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>Candidate - Semester A to confirm</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>City University of Hong Kong — Hong Kong (SAR)</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>SOES224 POLITICAL ECONOMIES OF CRISIS AND CHANGE (suggested)</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>PIA3126 International Political Economy (3 credit units)</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Level 3</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>CANDIDATE - on 2026/27 inbound exchange list (Semester B list); Semester A list not yet published - confirm Semester A</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="n"/>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>Host: https://banweb.cityu.edu.hk/pls/PROD/hwiecrselis_cityu.P_Main</t>
-        </is>
-      </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>Candidate - Semester A to confirm</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>City University of Hong Kong — Hong Kong (SAR)</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>SOES224 POLITICAL ECONOMIES OF CRISIS AND CHANGE (suggested)</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>PIA4152 Globalization and Its Discontents (3 credit units)</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Level 4</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>CANDIDATE - on 2026/27 inbound exchange list (Semester B list); Semester A list not yet published - confirm Semester A</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="n"/>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>Host: https://banweb.cityu.edu.hk/pls/PROD/hwiecrselis_cityu.P_Main</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>Candidate - Semester A to confirm</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>City University of Hong Kong — Hong Kong (SAR)</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY (suggested)</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>SEE3001 Energy and Environmental Policy (3 credit units)</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Level 3</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>CANDIDATE - on 2026/27 inbound exchange list (Semester B list); Semester A list not yet published - confirm Semester A</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="n"/>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>Host: https://banweb.cityu.edu.hk/pls/PROD/hwiecrselis_cityu.P_Main</t>
-        </is>
-      </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t>Candidate - Semester A to confirm</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>City University of Hong Kong — Hong Kong (SAR)</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY (suggested)</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>SEE3003 Climate Change and Adaptation Strategies (3 credit units)</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>Level 3</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>CANDIDATE - on 2026/27 inbound exchange list (Semester B list); Semester A list not yet published - confirm Semester A</t>
-        </is>
-      </c>
-      <c r="I8" s="4" t="n"/>
-      <c r="J8" s="4" t="inlineStr">
-        <is>
-          <t>Host: https://banweb.cityu.edu.hk/pls/PROD/hwiecrselis_cityu.P_Main</t>
-        </is>
-      </c>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>Candidate - Semester A to confirm</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>City University of Hong Kong — Hong Kong (SAR)</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>SOES226 EXPLORING THE SOCIAL WORLD (suggested)</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>SS3428 Advanced Applied Qualitative Research Methods (3 credit units)</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>Level 3</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>CANDIDATE - on 2026/27 inbound exchange list (Semester B list); Semester A list not yet published - confirm Semester A</t>
-        </is>
-      </c>
-      <c r="I9" s="4" t="n"/>
-      <c r="J9" s="4" t="inlineStr">
-        <is>
-          <t>Host: https://banweb.cityu.edu.hk/pls/PROD/hwiecrselis_cityu.P_Main</t>
-        </is>
-      </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>Candidate - Semester A to confirm</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>City University of Hong Kong — Hong Kong (SAR)</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>SOES225 THEMES IN URBAN GEOGRAPHY (suggested)</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>GE2339 Smart City - a Systems Engineering Perspective (3 credit units)</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>Level 2</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>CANDIDATE - on 2026/27 inbound exchange list (Semester B list); Semester A list not yet published - confirm Semester A</t>
-        </is>
-      </c>
-      <c r="I10" s="4" t="n"/>
-      <c r="J10" s="4" t="inlineStr">
-        <is>
-          <t>Host: https://banweb.cityu.edu.hk/pls/PROD/hwiecrselis_cityu.P_Main</t>
-        </is>
-      </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>Candidate - Semester A to confirm</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:K10"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
ACU BSc: Semester 1 unit check recorded
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EZa6h9SpqLeB7ZbHz6KiwN
</commit_message>
<xml_diff>
--- a/curriculum_mapping_2026-27/CurriculumMapping_Geo_2_ReviewEntry_NOT_met.xlsx
+++ b/curriculum_mapping_2026-27/CurriculumMapping_Geo_2_ReviewEntry_NOT_met.xlsx
@@ -47,7 +47,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -61,7 +61,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFE699"/>
+        <fgColor rgb="00F8CBAD"/>
       </patternFill>
     </fill>
     <fill>
@@ -73,11 +73,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E4DFEC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F8CBAD"/>
       </patternFill>
     </fill>
   </fills>
@@ -93,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -107,9 +102,6 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -574,7 +566,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Not enough modules after 2026/27 term check: 1 confirmed + 0 unverified, 4 needed</t>
+          <t>Not enough: ACU offers only 4 GEOG units in Semester 1 (2026 handbook: GEOG111, GEOG217, GEOG218, GEOG310) and only GEOG218 is physical; GEOG110/GEOG311 are Semester 2 only; other Semester 1 science units are human biology/biomedical. 1 usable for BSc, 4 needed. BSc could only reach 4 by taking the human-geography units used for the BA.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -897,212 +889,212 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Australian Catholic University — Australia</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Geography BSc</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>SOES214 CHANGING ENVIRONMENTS</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Level 5</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>GEOG110 Exploring Natural Environments (10 CP)</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>Level 1</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>Semester 2 (2026)</t>
         </is>
       </c>
-      <c r="I2" s="7" t="n"/>
-      <c r="J2" s="7" t="inlineStr">
+      <c r="I2" s="4" t="n"/>
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>Host: https://www.acu.edu.au/handbook/handbook-2026/major/geography-environment-and-society | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
         </is>
       </c>
-      <c r="K2" s="7" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>Original row; Wrong term for partner semester (Semester 1)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Australian Catholic University — Australia</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Geography BSc</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>SOES280 HYDROCLIMATE</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Level 5</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>GEOG216 Climate Change: Past, Present and Future (10 CP)</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>Level 2</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>Not listed in 2026 Geography, Environment and Society unit availability</t>
         </is>
       </c>
-      <c r="I3" s="7" t="n"/>
-      <c r="J3" s="7" t="inlineStr">
+      <c r="I3" s="4" t="n"/>
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>Host: https://www.acu.edu.au/handbook/handbook-2026/major/geography-environment-and-society | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
         </is>
       </c>
-      <c r="K3" s="7" t="inlineStr">
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>Original row; Workbook semester note says not currently offered</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Australian Catholic University — Australia</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Geography BSc</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>SOES280 HYDROCLIMATE</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Level 5</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>GEOG311 Catchments to Coasts (10 CP)</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Level 3</t>
         </is>
       </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Semester 2 (2026)</t>
         </is>
       </c>
-      <c r="I4" s="7" t="n"/>
-      <c r="J4" s="7" t="inlineStr">
+      <c r="I4" s="4" t="n"/>
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>Host: https://www.acu.edu.au/handbook/handbook-2026/major/geography-environment-and-society | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
         </is>
       </c>
-      <c r="K4" s="7" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>Original row; Wrong term for partner semester (Semester 1)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Australian Catholic University — Australia</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Geography BSc</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Level 5</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>GEOG312 Mapping for a Complex World (10 CP)</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Level 3</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Not listed in 2026 Geography, Environment and Society unit availability</t>
         </is>
       </c>
-      <c r="I5" s="7" t="n"/>
-      <c r="J5" s="7" t="inlineStr">
+      <c r="I5" s="4" t="n"/>
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>Host: https://www.acu.edu.au/handbook/handbook-2026/major/geography-environment-and-society | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
         </is>
       </c>
-      <c r="K5" s="7" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>Original row; Workbook semester note says not currently offered</t>
         </is>

</xml_diff>